<commit_message>
Prepare repository for public release
</commit_message>
<xml_diff>
--- a/data/metadata_raw/construction_output.xlsx
+++ b/data/metadata_raw/construction_output.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="1238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="1239">
   <si>
     <t>Code</t>
   </si>
@@ -2852,6 +2852,9 @@
     <t>Бухоро тумани</t>
   </si>
   <si>
+    <t>Вобкент тумани</t>
+  </si>
+  <si>
     <t>Ғиждувон тумани</t>
   </si>
   <si>
@@ -3596,7 +3599,7 @@
     <t>2023-01-13</t>
   </si>
   <si>
-    <t>2024-08-09</t>
+    <t>2025-11-13</t>
   </si>
   <si>
     <t>1.04.02.0001</t>
@@ -6720,7 +6723,7 @@
         <v>724</v>
       </c>
       <c r="E43" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="F43">
         <v>19</v>
@@ -6782,7 +6785,7 @@
         <v>725</v>
       </c>
       <c r="E44" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="F44">
         <v>37.2</v>
@@ -6844,7 +6847,7 @@
         <v>726</v>
       </c>
       <c r="E45" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="F45">
         <v>83</v>
@@ -6906,7 +6909,7 @@
         <v>727</v>
       </c>
       <c r="E46" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="F46">
         <v>23</v>
@@ -6968,7 +6971,7 @@
         <v>728</v>
       </c>
       <c r="E47" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="F47">
         <v>58.4</v>
@@ -7030,7 +7033,7 @@
         <v>729</v>
       </c>
       <c r="E48" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="F48">
         <v>17</v>
@@ -7092,7 +7095,7 @@
         <v>730</v>
       </c>
       <c r="E49" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="F49">
         <v>32.1</v>
@@ -7154,7 +7157,7 @@
         <v>731</v>
       </c>
       <c r="E50" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="F50">
         <v>23.4</v>
@@ -7216,7 +7219,7 @@
         <v>732</v>
       </c>
       <c r="E51" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="F51">
         <v>30</v>
@@ -7278,7 +7281,7 @@
         <v>733</v>
       </c>
       <c r="E52" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="F52">
         <v>211.5</v>
@@ -7340,7 +7343,7 @@
         <v>734</v>
       </c>
       <c r="E53" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="F53">
         <v>93.09999999999999</v>
@@ -7402,7 +7405,7 @@
         <v>735</v>
       </c>
       <c r="E54" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="F54">
         <v>2.5</v>
@@ -7464,7 +7467,7 @@
         <v>736</v>
       </c>
       <c r="E55" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="F55">
         <v>15.6</v>
@@ -7526,7 +7529,7 @@
         <v>737</v>
       </c>
       <c r="E56" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="F56">
         <v>13.7</v>
@@ -7588,7 +7591,7 @@
         <v>738</v>
       </c>
       <c r="E57" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="F57">
         <v>27.8</v>
@@ -7650,7 +7653,7 @@
         <v>739</v>
       </c>
       <c r="E58" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="F58">
         <v>6.7</v>
@@ -7712,7 +7715,7 @@
         <v>740</v>
       </c>
       <c r="E59" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="F59">
         <v>15.8</v>
@@ -7774,7 +7777,7 @@
         <v>741</v>
       </c>
       <c r="E60" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="F60">
         <v>6.8</v>
@@ -7836,7 +7839,7 @@
         <v>742</v>
       </c>
       <c r="E61" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="F61">
         <v>4.5</v>
@@ -7898,7 +7901,7 @@
         <v>743</v>
       </c>
       <c r="E62" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="F62">
         <v>2.2</v>
@@ -7960,7 +7963,7 @@
         <v>744</v>
       </c>
       <c r="E63" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="F63">
         <v>10.4</v>
@@ -8022,7 +8025,7 @@
         <v>745</v>
       </c>
       <c r="E64" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="F64">
         <v>9.699999999999999</v>
@@ -8084,7 +8087,7 @@
         <v>746</v>
       </c>
       <c r="E65" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="F65">
         <v>2.7</v>
@@ -8146,7 +8149,7 @@
         <v>747</v>
       </c>
       <c r="E66" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="F66">
         <v>699.2</v>
@@ -8208,7 +8211,7 @@
         <v>748</v>
       </c>
       <c r="E67" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="F67">
         <v>189.4</v>
@@ -8270,7 +8273,7 @@
         <v>749</v>
       </c>
       <c r="E68" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="F68">
         <v>0</v>
@@ -8332,7 +8335,7 @@
         <v>750</v>
       </c>
       <c r="E69" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="F69">
         <v>0</v>
@@ -8394,7 +8397,7 @@
         <v>751</v>
       </c>
       <c r="E70" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="F70">
         <v>89.2</v>
@@ -8456,7 +8459,7 @@
         <v>752</v>
       </c>
       <c r="E71" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="F71">
         <v>19.1</v>
@@ -8518,7 +8521,7 @@
         <v>753</v>
       </c>
       <c r="E72" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="F72">
         <v>23.6</v>
@@ -8580,7 +8583,7 @@
         <v>754</v>
       </c>
       <c r="E73" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="F73">
         <v>54.4</v>
@@ -8642,7 +8645,7 @@
         <v>755</v>
       </c>
       <c r="E74" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="F74">
         <v>55.1</v>
@@ -8704,7 +8707,7 @@
         <v>756</v>
       </c>
       <c r="E75" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="F75">
         <v>37.2</v>
@@ -8766,7 +8769,7 @@
         <v>757</v>
       </c>
       <c r="E76" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="F76">
         <v>18.6</v>
@@ -8828,7 +8831,7 @@
         <v>758</v>
       </c>
       <c r="E77" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="F77">
         <v>45.9</v>
@@ -8890,7 +8893,7 @@
         <v>759</v>
       </c>
       <c r="E78" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="F78">
         <v>24.4</v>
@@ -8952,7 +8955,7 @@
         <v>760</v>
       </c>
       <c r="E79" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="F79">
         <v>23.5</v>
@@ -9014,7 +9017,7 @@
         <v>761</v>
       </c>
       <c r="E80" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="F80">
         <v>26.6</v>
@@ -9076,7 +9079,7 @@
         <v>762</v>
       </c>
       <c r="E81" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="F81">
         <v>55.9</v>
@@ -9138,7 +9141,7 @@
         <v>763</v>
       </c>
       <c r="E82" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="F82">
         <v>36.3</v>
@@ -9200,7 +9203,7 @@
         <v>764</v>
       </c>
       <c r="E83" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="F83">
         <v>418.9</v>
@@ -9262,7 +9265,7 @@
         <v>765</v>
       </c>
       <c r="E84" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="F84">
         <v>84.90000000000001</v>
@@ -9324,7 +9327,7 @@
         <v>766</v>
       </c>
       <c r="E85" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="F85">
         <v>158.6</v>
@@ -9386,7 +9389,7 @@
         <v>767</v>
       </c>
       <c r="E86" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="F86">
         <v>0</v>
@@ -9448,7 +9451,7 @@
         <v>768</v>
       </c>
       <c r="E87" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="F87">
         <v>7.3</v>
@@ -9510,7 +9513,7 @@
         <v>769</v>
       </c>
       <c r="E88" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="F88">
         <v>53.6</v>
@@ -9572,7 +9575,7 @@
         <v>770</v>
       </c>
       <c r="E89" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="F89">
         <v>20</v>
@@ -9634,7 +9637,7 @@
         <v>771</v>
       </c>
       <c r="E90" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="F90">
         <v>44.4</v>
@@ -9696,7 +9699,7 @@
         <v>772</v>
       </c>
       <c r="E91" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="F91">
         <v>26.9</v>
@@ -9758,7 +9761,7 @@
         <v>773</v>
       </c>
       <c r="E92" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="F92">
         <v>2.5</v>
@@ -9820,7 +9823,7 @@
         <v>774</v>
       </c>
       <c r="E93" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="F93">
         <v>4.6</v>
@@ -9882,7 +9885,7 @@
         <v>775</v>
       </c>
       <c r="E94" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="F94">
         <v>16.1</v>
@@ -9944,7 +9947,7 @@
         <v>776</v>
       </c>
       <c r="E95" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="F95">
         <v>347.9</v>
@@ -10006,7 +10009,7 @@
         <v>777</v>
       </c>
       <c r="E96" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="F96">
         <v>84.09999999999999</v>
@@ -10068,7 +10071,7 @@
         <v>778</v>
       </c>
       <c r="E97" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="F97">
         <v>12.2</v>
@@ -10130,7 +10133,7 @@
         <v>779</v>
       </c>
       <c r="E98" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="F98">
         <v>23.6</v>
@@ -10192,7 +10195,7 @@
         <v>780</v>
       </c>
       <c r="E99" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="F99">
         <v>34.9</v>
@@ -10254,7 +10257,7 @@
         <v>781</v>
       </c>
       <c r="E100" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="F100">
         <v>14.9</v>
@@ -10316,7 +10319,7 @@
         <v>782</v>
       </c>
       <c r="E101" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="F101">
         <v>28.5</v>
@@ -10378,7 +10381,7 @@
         <v>783</v>
       </c>
       <c r="E102" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="F102">
         <v>26.8</v>
@@ -10440,7 +10443,7 @@
         <v>784</v>
       </c>
       <c r="E103" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="F103">
         <v>31.1</v>
@@ -10502,7 +10505,7 @@
         <v>785</v>
       </c>
       <c r="E104" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="F104">
         <v>16.5</v>
@@ -10564,7 +10567,7 @@
         <v>786</v>
       </c>
       <c r="E105" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="F105">
         <v>26.5</v>
@@ -10626,7 +10629,7 @@
         <v>787</v>
       </c>
       <c r="E106" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="F106">
         <v>26.1</v>
@@ -10688,7 +10691,7 @@
         <v>788</v>
       </c>
       <c r="E107" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="F107">
         <v>22.7</v>
@@ -10750,7 +10753,7 @@
         <v>789</v>
       </c>
       <c r="E108" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="F108">
         <v>519.7</v>
@@ -10812,7 +10815,7 @@
         <v>790</v>
       </c>
       <c r="E109" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="F109">
         <v>200.3</v>
@@ -10874,7 +10877,7 @@
         <v>791</v>
       </c>
       <c r="E110" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="F110">
         <v>8.6</v>
@@ -10936,7 +10939,7 @@
         <v>792</v>
       </c>
       <c r="E111" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="F111">
         <v>28.2</v>
@@ -10998,7 +11001,7 @@
         <v>793</v>
       </c>
       <c r="E112" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="F112">
         <v>14.3</v>
@@ -11060,7 +11063,7 @@
         <v>794</v>
       </c>
       <c r="E113" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="F113">
         <v>20.3</v>
@@ -11122,7 +11125,7 @@
         <v>795</v>
       </c>
       <c r="E114" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="F114">
         <v>17.3</v>
@@ -11184,7 +11187,7 @@
         <v>796</v>
       </c>
       <c r="E115" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="F115">
         <v>21.8</v>
@@ -11246,7 +11249,7 @@
         <v>797</v>
       </c>
       <c r="E116" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="F116">
         <v>14.4</v>
@@ -11308,7 +11311,7 @@
         <v>798</v>
       </c>
       <c r="E117" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="F117">
         <v>25</v>
@@ -11370,7 +11373,7 @@
         <v>799</v>
       </c>
       <c r="E118" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="F118">
         <v>22.1</v>
@@ -11432,7 +11435,7 @@
         <v>800</v>
       </c>
       <c r="E119" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="F119">
         <v>28</v>
@@ -11494,7 +11497,7 @@
         <v>801</v>
       </c>
       <c r="E120" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="F120">
         <v>14.7</v>
@@ -11556,7 +11559,7 @@
         <v>802</v>
       </c>
       <c r="E121" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="F121">
         <v>41</v>
@@ -11618,7 +11621,7 @@
         <v>803</v>
       </c>
       <c r="E122" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="F122">
         <v>13.1</v>
@@ -11680,7 +11683,7 @@
         <v>804</v>
       </c>
       <c r="E123" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="F123">
         <v>30.7</v>
@@ -11742,7 +11745,7 @@
         <v>805</v>
       </c>
       <c r="E124" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="F124">
         <v>19.9</v>
@@ -11804,7 +11807,7 @@
         <v>806</v>
       </c>
       <c r="E125" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="F125">
         <v>335.9</v>
@@ -11866,7 +11869,7 @@
         <v>807</v>
       </c>
       <c r="E126" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="F126">
         <v>66.59999999999999</v>
@@ -11928,7 +11931,7 @@
         <v>808</v>
       </c>
       <c r="E127" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="F127">
         <v>14</v>
@@ -11990,7 +11993,7 @@
         <v>809</v>
       </c>
       <c r="E128" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="F128">
         <v>12.4</v>
@@ -12052,7 +12055,7 @@
         <v>810</v>
       </c>
       <c r="E129" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="F129">
         <v>10.4</v>
@@ -12114,7 +12117,7 @@
         <v>811</v>
       </c>
       <c r="E130" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="F130">
         <v>24.9</v>
@@ -12176,7 +12179,7 @@
         <v>812</v>
       </c>
       <c r="E131" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="F131">
         <v>13.3</v>
@@ -12238,7 +12241,7 @@
         <v>813</v>
       </c>
       <c r="E132" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="F132">
         <v>30.7</v>
@@ -12300,7 +12303,7 @@
         <v>814</v>
       </c>
       <c r="E133" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="F133">
         <v>23.9</v>
@@ -12362,7 +12365,7 @@
         <v>815</v>
       </c>
       <c r="E134" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="F134">
         <v>17.5</v>
@@ -12424,7 +12427,7 @@
         <v>816</v>
       </c>
       <c r="E135" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="F135">
         <v>11</v>
@@ -12486,7 +12489,7 @@
         <v>817</v>
       </c>
       <c r="E136" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="F136">
         <v>43.7</v>
@@ -12548,7 +12551,7 @@
         <v>818</v>
       </c>
       <c r="E137" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="F137">
         <v>16.4</v>
@@ -12610,7 +12613,7 @@
         <v>819</v>
       </c>
       <c r="E138" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F138">
         <v>18.6</v>
@@ -12672,7 +12675,7 @@
         <v>820</v>
       </c>
       <c r="E139" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="F139">
         <v>20.5</v>
@@ -12734,7 +12737,7 @@
         <v>821</v>
       </c>
       <c r="E140" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="F140">
         <v>12</v>
@@ -12796,7 +12799,7 @@
         <v>822</v>
       </c>
       <c r="E141" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="F141">
         <v>134.9</v>
@@ -12858,7 +12861,7 @@
         <v>823</v>
       </c>
       <c r="E142" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="F142">
         <v>34.4</v>
@@ -12920,7 +12923,7 @@
         <v>824</v>
       </c>
       <c r="E143" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="F143">
         <v>3.9</v>
@@ -12982,7 +12985,7 @@
         <v>825</v>
       </c>
       <c r="E144" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="F144">
         <v>7.9</v>
@@ -13044,7 +13047,7 @@
         <v>826</v>
       </c>
       <c r="E145" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F145">
         <v>3.6</v>
@@ -13106,7 +13109,7 @@
         <v>827</v>
       </c>
       <c r="E146" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F146">
         <v>13.1</v>
@@ -13168,7 +13171,7 @@
         <v>828</v>
       </c>
       <c r="E147" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="F147">
         <v>7.8</v>
@@ -13230,7 +13233,7 @@
         <v>829</v>
       </c>
       <c r="E148" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="F148">
         <v>9.9</v>
@@ -13292,7 +13295,7 @@
         <v>830</v>
       </c>
       <c r="E149" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="F149">
         <v>6</v>
@@ -13354,7 +13357,7 @@
         <v>831</v>
       </c>
       <c r="E150" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="F150">
         <v>11.1</v>
@@ -13416,7 +13419,7 @@
         <v>832</v>
       </c>
       <c r="E151" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="F151">
         <v>28.6</v>
@@ -13478,7 +13481,7 @@
         <v>833</v>
       </c>
       <c r="E152" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="F152">
         <v>8.800000000000001</v>
@@ -13540,7 +13543,7 @@
         <v>834</v>
       </c>
       <c r="E153" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="F153">
         <v>509.9</v>
@@ -13602,7 +13605,7 @@
         <v>835</v>
       </c>
       <c r="E154" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="F154">
         <v>0</v>
@@ -13664,7 +13667,7 @@
         <v>836</v>
       </c>
       <c r="E155" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="F155">
         <v>62.7</v>
@@ -13726,7 +13729,7 @@
         <v>837</v>
       </c>
       <c r="E156" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="F156">
         <v>60.5</v>
@@ -13788,7 +13791,7 @@
         <v>838</v>
       </c>
       <c r="E157" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="F157">
         <v>17.6</v>
@@ -13850,7 +13853,7 @@
         <v>839</v>
       </c>
       <c r="E158" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="F158">
         <v>29.2</v>
@@ -13912,7 +13915,7 @@
         <v>840</v>
       </c>
       <c r="E159" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="F159">
         <v>0</v>
@@ -13974,7 +13977,7 @@
         <v>841</v>
       </c>
       <c r="E160" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="F160">
         <v>0</v>
@@ -14036,7 +14039,7 @@
         <v>842</v>
       </c>
       <c r="E161" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="F161">
         <v>9.9</v>
@@ -14098,7 +14101,7 @@
         <v>843</v>
       </c>
       <c r="E162" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="F162">
         <v>17.4</v>
@@ -14160,7 +14163,7 @@
         <v>844</v>
       </c>
       <c r="E163" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="F163">
         <v>12.9</v>
@@ -14222,7 +14225,7 @@
         <v>845</v>
       </c>
       <c r="E164" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="F164">
         <v>38.2</v>
@@ -14284,7 +14287,7 @@
         <v>846</v>
       </c>
       <c r="E165" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="F165">
         <v>10.8</v>
@@ -14346,7 +14349,7 @@
         <v>847</v>
       </c>
       <c r="E166" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="F166">
         <v>6.9</v>
@@ -14408,7 +14411,7 @@
         <v>848</v>
       </c>
       <c r="E167" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="F167">
         <v>66.59999999999999</v>
@@ -14470,7 +14473,7 @@
         <v>849</v>
       </c>
       <c r="E168" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="F168">
         <v>37.5</v>
@@ -14532,7 +14535,7 @@
         <v>850</v>
       </c>
       <c r="E169" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="F169">
         <v>54</v>
@@ -14594,7 +14597,7 @@
         <v>851</v>
       </c>
       <c r="E170" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="F170">
         <v>13.8</v>
@@ -14656,7 +14659,7 @@
         <v>852</v>
       </c>
       <c r="E171" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="F171">
         <v>8.9</v>
@@ -14718,7 +14721,7 @@
         <v>853</v>
       </c>
       <c r="E172" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="F172">
         <v>10</v>
@@ -14780,7 +14783,7 @@
         <v>854</v>
       </c>
       <c r="E173" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="F173">
         <v>14.9</v>
@@ -14842,7 +14845,7 @@
         <v>855</v>
       </c>
       <c r="E174" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="F174">
         <v>38.3</v>
@@ -14904,7 +14907,7 @@
         <v>856</v>
       </c>
       <c r="E175" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="F175">
         <v>0</v>
@@ -14966,7 +14969,7 @@
         <v>857</v>
       </c>
       <c r="E176" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F176">
         <v>489.2</v>
@@ -15028,7 +15031,7 @@
         <v>858</v>
       </c>
       <c r="E177" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="F177">
         <v>100.4</v>
@@ -15090,7 +15093,7 @@
         <v>859</v>
       </c>
       <c r="E178" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="F178">
         <v>49.6</v>
@@ -15152,7 +15155,7 @@
         <v>860</v>
       </c>
       <c r="E179" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="F179">
         <v>23.4</v>
@@ -15214,7 +15217,7 @@
         <v>861</v>
       </c>
       <c r="E180" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F180">
         <v>22.2</v>
@@ -15276,7 +15279,7 @@
         <v>862</v>
       </c>
       <c r="E181" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="F181">
         <v>35.4</v>
@@ -15338,7 +15341,7 @@
         <v>863</v>
       </c>
       <c r="E182" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="F182">
         <v>13.1</v>
@@ -15400,7 +15403,7 @@
         <v>864</v>
       </c>
       <c r="E183" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="F183">
         <v>20.1</v>
@@ -15462,7 +15465,7 @@
         <v>865</v>
       </c>
       <c r="E184" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="F184">
         <v>13.9</v>
@@ -15524,7 +15527,7 @@
         <v>866</v>
       </c>
       <c r="E185" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="F185">
         <v>16.9</v>
@@ -15586,7 +15589,7 @@
         <v>867</v>
       </c>
       <c r="E186" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="F186">
         <v>25.2</v>
@@ -15648,7 +15651,7 @@
         <v>868</v>
       </c>
       <c r="E187" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="F187">
         <v>18.4</v>
@@ -15710,7 +15713,7 @@
         <v>869</v>
       </c>
       <c r="E188" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="F188">
         <v>19.3</v>
@@ -15772,7 +15775,7 @@
         <v>870</v>
       </c>
       <c r="E189" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="F189">
         <v>11.3</v>
@@ -15834,7 +15837,7 @@
         <v>871</v>
       </c>
       <c r="E190" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="F190">
         <v>16.6</v>
@@ -15896,7 +15899,7 @@
         <v>872</v>
       </c>
       <c r="E191" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="F191">
         <v>19.7</v>
@@ -15958,7 +15961,7 @@
         <v>873</v>
       </c>
       <c r="E192" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="F192">
         <v>24.7</v>
@@ -16020,7 +16023,7 @@
         <v>874</v>
       </c>
       <c r="E193" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="F193">
         <v>27.4</v>
@@ -16082,7 +16085,7 @@
         <v>875</v>
       </c>
       <c r="E194" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="F194">
         <v>11.6</v>
@@ -16144,7 +16147,7 @@
         <v>876</v>
       </c>
       <c r="E195" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="F195">
         <v>20</v>
@@ -16206,7 +16209,7 @@
         <v>877</v>
       </c>
       <c r="E196" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="F196">
         <v>282.7</v>
@@ -16268,7 +16271,7 @@
         <v>878</v>
       </c>
       <c r="E197" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="F197">
         <v>69.40000000000001</v>
@@ -16330,7 +16333,7 @@
         <v>879</v>
       </c>
       <c r="E198" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="F198">
         <v>0</v>
@@ -16392,7 +16395,7 @@
         <v>880</v>
       </c>
       <c r="E199" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="F199">
         <v>16.4</v>
@@ -16454,7 +16457,7 @@
         <v>881</v>
       </c>
       <c r="E200" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="F200">
         <v>14.9</v>
@@ -16516,7 +16519,7 @@
         <v>882</v>
       </c>
       <c r="E201" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="F201">
         <v>13.6</v>
@@ -16578,7 +16581,7 @@
         <v>883</v>
       </c>
       <c r="E202" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="F202">
         <v>27.5</v>
@@ -16640,7 +16643,7 @@
         <v>884</v>
       </c>
       <c r="E203" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="F203">
         <v>22.1</v>
@@ -16702,7 +16705,7 @@
         <v>885</v>
       </c>
       <c r="E204" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="F204">
         <v>0</v>
@@ -16764,7 +16767,7 @@
         <v>886</v>
       </c>
       <c r="E205" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="F205">
         <v>22.2</v>
@@ -16826,7 +16829,7 @@
         <v>887</v>
       </c>
       <c r="E206" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="F206">
         <v>50</v>
@@ -16888,7 +16891,7 @@
         <v>888</v>
       </c>
       <c r="E207" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="F207">
         <v>18.4</v>
@@ -16950,7 +16953,7 @@
         <v>889</v>
       </c>
       <c r="E208" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="F208">
         <v>13.3</v>
@@ -17012,7 +17015,7 @@
         <v>890</v>
       </c>
       <c r="E209" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="F209">
         <v>14.6</v>
@@ -17074,7 +17077,7 @@
         <v>891</v>
       </c>
       <c r="E210" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="F210">
         <v>1228.4</v>
@@ -17136,7 +17139,7 @@
         <v>892</v>
       </c>
       <c r="E211" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="F211">
         <v>33.2</v>
@@ -17198,7 +17201,7 @@
         <v>893</v>
       </c>
       <c r="E212" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="F212">
         <v>53.2</v>
@@ -17260,7 +17263,7 @@
         <v>894</v>
       </c>
       <c r="E213" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="F213">
         <v>90.09999999999999</v>
@@ -17322,7 +17325,7 @@
         <v>895</v>
       </c>
       <c r="E214" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="F214">
         <v>98.59999999999999</v>
@@ -17384,7 +17387,7 @@
         <v>896</v>
       </c>
       <c r="E215" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="F215">
         <v>173.4</v>
@@ -17446,7 +17449,7 @@
         <v>897</v>
       </c>
       <c r="E216" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="F216">
         <v>133.3</v>
@@ -17508,7 +17511,7 @@
         <v>898</v>
       </c>
       <c r="E217" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="F217">
         <v>45.5</v>
@@ -17570,7 +17573,7 @@
         <v>899</v>
       </c>
       <c r="E218" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="F218">
         <v>52.5</v>
@@ -17632,7 +17635,7 @@
         <v>900</v>
       </c>
       <c r="E219" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="F219">
         <v>80.59999999999999</v>
@@ -17694,7 +17697,7 @@
         <v>901</v>
       </c>
       <c r="E220" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="F220">
         <v>78.3</v>
@@ -17756,7 +17759,7 @@
         <v>902</v>
       </c>
       <c r="E221" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="F221">
         <v>0</v>
@@ -17818,7 +17821,7 @@
         <v>903</v>
       </c>
       <c r="E222" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="F222">
         <v>389.7</v>
@@ -17878,444 +17881,444 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B2" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="C2" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="D2" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="E2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="F2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="G2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="H2" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B3" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="C3" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="D3" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="E3" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="F3" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="G3" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="H3" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="B4" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="C4" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="D4" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="E4" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="F4" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="G4" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="H4" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="B5" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="C5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="D5" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="E5" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="F5" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="G5" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="H5" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B6" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="C6" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="D6" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="E6" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="F6" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="G6" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="H6" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="B7" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="C7" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="D7" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="E7" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="F7" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="G7" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="H7" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="B8" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="C8" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="D8" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B9" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="C9" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="D9" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="E9" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="F9" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="G9" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="H9" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="B10" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="C10" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="D10" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="E10" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="F10" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="G10" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="H10" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="B11" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="C11" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="D11" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="E11" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="F11" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="G11" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="H11" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B12" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="C12" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="D12" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="E12" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="F12" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="G12" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="H12" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="B13" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C13" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="D13" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="E13" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="F13" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="G13" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="H13" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="B14" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="C14" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="D14" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="E14" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="F14" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="G14" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="H14" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B15" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="C15" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="D15" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="E15" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="F15" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="G15" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="H15" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="B16" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="C16" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="D16" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="E16" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="F16" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="G16" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="H16" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="B17" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="C17" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="D17" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="E17" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="F17" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="G17" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="H17" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>